<commit_message>
still working on changes
</commit_message>
<xml_diff>
--- a/rules/CORE-000726/negative/01/data/unit-test-coreid-FB5701-negative_01.xlsx
+++ b/rules/CORE-000726/negative/01/data/unit-test-coreid-FB5701-negative_01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\verisian\core-contributor\rules\CORE-000726\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{669511D1-6D58-4C04-8CA0-AD3E961EC089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01D4A660-DCA1-4D69-BF8C-A6BCDDDC0FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="99">
   <si>
     <t>Product</t>
   </si>
@@ -305,9 +305,6 @@
   </si>
   <si>
     <t>Evaluator</t>
-  </si>
-  <si>
-    <t>CDISC-TEST</t>
   </si>
   <si>
     <t>CETHNIC</t>
@@ -472,7 +469,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -874,7 +871,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D2">
         <v>5</v>
@@ -894,13 +891,13 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D3">
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F3" s="10"/>
     </row>
@@ -912,7 +909,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D4">
         <v>5</v>
@@ -921,7 +918,7 @@
         <v>82</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -932,7 +929,7 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D5">
         <v>7</v>
@@ -952,13 +949,13 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D6">
         <v>7</v>
       </c>
       <c r="E6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F6" s="10"/>
     </row>
@@ -970,7 +967,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D7">
         <v>7</v>
@@ -979,7 +976,7 @@
         <v>82</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -990,7 +987,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D8">
         <v>8</v>
@@ -1010,13 +1007,13 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D9">
         <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F9" s="10"/>
     </row>
@@ -1028,7 +1025,7 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D10">
         <v>8</v>
@@ -1037,7 +1034,7 @@
         <v>82</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -1539,8 +1536,8 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
-        <v>93</v>
+      <c r="A5" s="9" t="s">
+        <v>46</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>47</v>
@@ -1549,21 +1546,21 @@
         <v>59</v>
       </c>
       <c r="F5" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="G5" s="10" t="s">
         <v>94</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>95</v>
       </c>
       <c r="H5" s="10" t="s">
         <v>58</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>93</v>
+      <c r="A6" s="9" t="s">
+        <v>46</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>47</v>
@@ -1572,33 +1569,39 @@
         <v>71</v>
       </c>
       <c r="F6" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="G6" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="H6" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="I6" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="H6" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="I6" s="13" t="s">
-        <v>96</v>
-      </c>
     </row>
     <row r="7" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
+        <v>46</v>
+      </c>
       <c r="C7" s="13" t="s">
         <v>66</v>
       </c>
       <c r="F7" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="G7" s="10" t="s">
         <v>94</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>95</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>46</v>
+      </c>
       <c r="C8" s="13" t="s">
         <v>48</v>
       </c>

</xml_diff>